<commit_message>
Refresh Google Search planning evidence
</commit_message>
<xml_diff>
--- a/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
+++ b/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="Red108f82ec0f4e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="R7cefd754d00449a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R309ea082219f4c61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="R54ef603b27094317"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -256,7 +256,7 @@
         <x:color rgb="FF0F766E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F3EF"/>
         </x:patternFill>
       </x:fill>
@@ -267,7 +267,7 @@
         <x:color rgb="FFA32C2A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -278,7 +278,7 @@
         <x:color rgb="FF8A5A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -289,7 +289,7 @@
         <x:color rgb="FF315D83"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1F8"/>
         </x:patternFill>
       </x:fill>
@@ -300,7 +300,7 @@
         <x:color rgb="FF0F766E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F3EF"/>
         </x:patternFill>
       </x:fill>
@@ -311,7 +311,7 @@
         <x:color rgb="FF315D83"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1F8"/>
         </x:patternFill>
       </x:fill>
@@ -322,7 +322,7 @@
         <x:color rgb="FFA32C2A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -333,7 +333,7 @@
         <x:color rgb="FF8A5A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
@@ -832,7 +832,7 @@
     </x:row>
     <x:row r="21" ht="36" hidden="0" customHeight="1">
       <x:c r="A21" s="34" t="str">
-        <x:v>Fresh Vietnam Keyword Planner research</x:v>
+        <x:v>Nghiên cứu Google Keyword Planner tại Việt Nam</x:v>
       </x:c>
       <x:c r="B21" s="34" t="str">
         <x:v>Bị kẹt</x:v>
@@ -843,7 +843,7 @@
 D:\Digiwin_Semiconducter_Workspace\operations\Pre_Ad_UI_Validation_Evidence.md</x:v>
       </x:c>
       <x:c r="D21" s="42" t="str">
-        <x:v>A visible “Turn off ad blockers” modal stopped work at Google Ads Overview; its effect beyond Overview is unknown. The orange mechanism-update banner is informational, not this blocker.</x:v>
+        <x:v>Một truy vấn OSAT không hiển thị metric; ảnh xác nhận Planner hoạt động, chuỗi ad-blocker chỉ có trong DOM. Yêu cầu kết quả tự tạo kế hoạch nháp; đã dừng hai cụm còn lại.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
@@ -932,8 +932,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68a721af2ee14bac"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c9fb7dd0bac484f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d394e696d574793"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeeea6c6caca4b15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1389,10 +1389,10 @@
         <x:v>D:\Digiwin_Semiconducter_Workspace\drafts\S02_Google_Search_Research.md</x:v>
       </x:c>
       <x:c r="G20" s="42" t="str">
-        <x:v>Fresh VN/Fabless/Partner Keyword Planner research is pending; current visible modal was at Overview.</x:v>
+        <x:v>Planner mở và truy vấn được. Cấu hình: Việt Nam, Tiếng Việt, Google, 09/2025–08/2026; loại trừ ý tưởng người lớn. Một truy vấn cho cụm OSAT hiển thị dấu gạch ngang ở mọi metric và không có dữ liệu biểu đồ/ý tưởng liên quan. Không suy luận nhu cầu bằng 0.</x:v>
       </x:c>
       <x:c r="H20" s="42" t="str">
-        <x:v>Resume only through an authorized route; modal effect beyond Overview is unknown.</x:v>
+        <x:v>Ảnh không có dialog ad-blocker; chuỗi còn trong DOM nhưng thao tác thành công. Lấy kết quả tự tạo một mục kế hoạch nháp dù không bấm lưu; đã dừng, chưa truy vấn Fabless và ERP–MES–OT/partner. Campaign chưa tạo/bật và chưa chi tiêu.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
@@ -1638,7 +1638,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R410a917f02304bf7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b16377dfc44f52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct Planner blocker evidence classification
</commit_message>
<xml_diff>
--- a/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
+++ b/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R309ea082219f4c61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="R54ef603b27094317"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R6aafdaa7c2164e0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="R863492cf1d144af4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -843,7 +843,7 @@
 D:\Digiwin_Semiconducter_Workspace\operations\Pre_Ad_UI_Validation_Evidence.md</x:v>
       </x:c>
       <x:c r="D21" s="42" t="str">
-        <x:v>Một truy vấn OSAT không hiển thị metric; ảnh xác nhận Planner hoạt động, chuỗi ad-blocker chỉ có trong DOM. Yêu cầu kết quả tự tạo kế hoạch nháp; đã dừng hai cụm còn lại.</x:v>
+        <x:v>Chuỗi ad-blocker chỉ có trong DOM/accessibility; ảnh không có dialog và thao tác Planner hoạt động. Một truy vấn OSAT không hiển thị metric, đồng thời tự tạo mục kế hoạch nháp. Chờ quyết định/mandate về việc chấp nhận các mục Planner tự tạo trước khi truy vấn thêm; đây là gate phạm vi/tác động phụ, không phải lỗi ad-blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
@@ -932,8 +932,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d394e696d574793"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeeea6c6caca4b15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4c81a12b0b4fdb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95aa044eebe4f9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1392,7 +1392,7 @@
         <x:v>Planner mở và truy vấn được. Cấu hình: Việt Nam, Tiếng Việt, Google, 09/2025–08/2026; loại trừ ý tưởng người lớn. Một truy vấn cho cụm OSAT hiển thị dấu gạch ngang ở mọi metric và không có dữ liệu biểu đồ/ý tưởng liên quan. Không suy luận nhu cầu bằng 0.</x:v>
       </x:c>
       <x:c r="H20" s="42" t="str">
-        <x:v>Ảnh không có dialog ad-blocker; chuỗi còn trong DOM nhưng thao tác thành công. Lấy kết quả tự tạo một mục kế hoạch nháp dù không bấm lưu; đã dừng, chưa truy vấn Fabless và ERP–MES–OT/partner. Campaign chưa tạo/bật và chưa chi tiêu.</x:v>
+        <x:v>Đính chính theo Bảo: chuỗi ad-blocker chỉ là false signal trong DOM/accessibility, không phải dialog từng hiển thị. Planner hoạt động. Lấy kết quả tự tạo một mục kế hoạch nháp dù không bấm lưu; chờ quyết định/mandate về việc chấp nhận thêm mục tự tạo trước truy vấn Fabless và ERP–MES–OT/partner. Đây là gate phạm vi/tác động phụ, không phải lỗi nền tảng. Campaign chưa tạo/bật và chưa chi tiêu.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
@@ -1638,7 +1638,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b16377dfc44f52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30bdd29fb6f24f5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record completed Keyword Planner cluster research
</commit_message>
<xml_diff>
--- a/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
+++ b/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R6aafdaa7c2164e0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="R863492cf1d144af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R61b8d9c6cc5a4a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="R1b2192aa96d34aad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -642,7 +642,7 @@
     <x:row r="6">
       <x:c r="A6" s="24" t="n">
         <x:f>COUNTIF('Asset inventory'!$E$6:$E$29,"Hoàn tất")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B6" s="24" t="n">
         <x:f>COUNTIF('Asset inventory'!$E$6:$E$29,"Đang thực hiện")</x:f>
@@ -650,7 +650,7 @@
       </x:c>
       <x:c r="C6" s="24" t="n">
         <x:f>COUNTIF('Asset inventory'!$E$6:$E$29,"Bị kẹt")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="24" t="n">
         <x:f>COUNTIF('Asset inventory'!$E$6:$E$29,"Hoãn")</x:f>
@@ -835,7 +835,7 @@
         <x:v>Nghiên cứu Google Keyword Planner tại Việt Nam</x:v>
       </x:c>
       <x:c r="B21" s="34" t="str">
-        <x:v>Bị kẹt</x:v>
+        <x:v>Hoàn tất</x:v>
       </x:c>
       <x:c r="C21" s="42" t="str">
         <x:v>D:\Digiwin_Semiconducter_Workspace\drafts\S02_Google_Search_Research.md
@@ -843,7 +843,7 @@
 D:\Digiwin_Semiconducter_Workspace\operations\Pre_Ad_UI_Validation_Evidence.md</x:v>
       </x:c>
       <x:c r="D21" s="42" t="str">
-        <x:v>Chuỗi ad-blocker chỉ có trong DOM/accessibility; ảnh không có dialog và thao tác Planner hoạt động. Một truy vấn OSAT không hiển thị metric, đồng thời tự tạo mục kế hoạch nháp. Chờ quyết định/mandate về việc chấp nhận các mục Planner tự tạo trước khi truy vấn thêm; đây là gate phạm vi/tác động phụ, không phải lỗi ad-blocker.</x:v>
+        <x:v>DOM-only ad-blocker text was a false signal; Planner interaction worked. OSAT/Fabless showed no displayed metrics; Partner had only one limited historical estimate and seven all-dash rows. Three automatic Planner drafts accepted; no campaign or spend. Broader account/campaign settings and performance remain unknown.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
@@ -932,8 +932,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4c81a12b0b4fdb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95aa044eebe4f9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9c44c9bc8a24976"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R935b52edfa8a4516"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1383,16 +1383,16 @@
         <x:v>Planning draft — Search keyword research</x:v>
       </x:c>
       <x:c r="E20" s="34" t="str">
-        <x:v>Bị kẹt</x:v>
+        <x:v>Hoàn tất</x:v>
       </x:c>
       <x:c r="F20" s="34" t="str">
         <x:v>D:\Digiwin_Semiconducter_Workspace\drafts\S02_Google_Search_Research.md</x:v>
       </x:c>
       <x:c r="G20" s="42" t="str">
-        <x:v>Planner mở và truy vấn được. Cấu hình: Việt Nam, Tiếng Việt, Google, 09/2025–08/2026; loại trừ ý tưởng người lớn. Một truy vấn cho cụm OSAT hiển thị dấu gạch ngang ở mọi metric và không có dữ liệu biểu đồ/ý tưởng liên quan. Không suy luận nhu cầu bằng 0.</x:v>
+        <x:v>Planner opened and all three planned Vietnamese-first seed clusters queried on 2026-09-14: OSAT and Fabless all displayed dashes; Partner had one row with 10 average monthly searches, 0% 3-month change and -100% year-over-year, seven all-dash rows. Dashes do not mean zero demand; one estimate is not a forecast or delivery result.</x:v>
       </x:c>
       <x:c r="H20" s="42" t="str">
-        <x:v>Đính chính theo Bảo: chuỗi ad-blocker chỉ là false signal trong DOM/accessibility, không phải dialog từng hiển thị. Planner hoạt động. Lấy kết quả tự tạo một mục kế hoạch nháp dù không bấm lưu; chờ quyết định/mandate về việc chấp nhận thêm mục tự tạo trước truy vấn Fabless và ERP–MES–OT/partner. Đây là gate phạm vi/tác động phụ, không phải lỗi nền tảng. Campaign chưa tạo/bật và chưa chi tiêu.</x:v>
+        <x:v>Research slice complete. Bảo accepted the three automatically created Planner draft entries; these are not campaigns. Metric ambiguity/low observed data leaves account overlap, live settings, CPC/competition and demand unresolved. No build, enablement or spend authorized by this evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
@@ -1638,7 +1638,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30bdd29fb6f24f5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28dba6d7bf9d424d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record sanitized LinkedIn validation handoff
</commit_message>
<xml_diff>
--- a/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
+++ b/outputs/01a08f67-5225-7ed1-bfb3-3c81ae70c25b/Digiwin_Semiconductor_Paid_Asset_Status.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R61b8d9c6cc5a4a43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="R1b2192aa96d34aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R0704242ef1d04cb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset inventory" sheetId="2" r:id="Rbc48267eaadb44a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -608,7 +608,7 @@
         <x:v>Nguồn</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
-        <x:v>Nhánh main chuẩn 141118e</x:v>
+        <x:v>Nhánh main chuẩn a518e80 trước đồng bộ LinkedIn</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -646,7 +646,7 @@
       </x:c>
       <x:c r="B6" s="24" t="n">
         <x:f>COUNTIF('Asset inventory'!$E$6:$E$29,"Đang thực hiện")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="24" t="n">
         <x:f>COUNTIF('Asset inventory'!$E$6:$E$29,"Bị kẹt")</x:f>
@@ -654,7 +654,7 @@
       </x:c>
       <x:c r="D6" s="24" t="n">
         <x:f>COUNTIF('Asset inventory'!$E$6:$E$29,"Hoãn")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -866,14 +866,14 @@
         <x:v>LinkedIn account, Page and placement verification</x:v>
       </x:c>
       <x:c r="B23" s="34" t="str">
-        <x:v>Bị kẹt</x:v>
+        <x:v>Hoàn tất</x:v>
       </x:c>
       <x:c r="C23" s="42" t="str">
         <x:v>D:\Digiwin_Semiconducter_Workspace\ads\linkedin\LinkedIn_Build_Pack.md
 D:\Digiwin_Semiconducter_Workspace\drafts\S03_LinkedIn_Audience_Research.md</x:v>
       </x:c>
       <x:c r="D23" s="42" t="str">
-        <x:v>Latest direct route redirected to sign-in. Account, Page and placement are not verified; no credentials were entered.</x:v>
+        <x:v>Đã có xác minh read-only bên ngoài repo (14-09-2026). Không upload, creative attach, delivery hoặc spend; proof raw không đưa vào public Git.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" hidden="0" customHeight="1">
@@ -881,14 +881,14 @@
         <x:v>LinkedIn audience and retargeting work</x:v>
       </x:c>
       <x:c r="B24" s="33" t="str">
-        <x:v>Hoãn</x:v>
+        <x:v>Đang thực hiện</x:v>
       </x:c>
       <x:c r="C24" s="41" t="str">
         <x:v>D:\Digiwin_Semiconducter_Workspace\drafts\S03_LinkedIn_Audience_Research.md
 D:\Digiwin_Semiconducter_Workspace\operations\Pre_Ad_Readiness_Plan.md</x:v>
       </x:c>
       <x:c r="D24" s="41" t="str">
-        <x:v>Deferred by Bảo. No audience upload. Retargeting remains conditional on evidence of at least 300 reachable members.</x:v>
+        <x:v>Xác minh external đã hoàn tất ở mức cấu hình; audience và retargeting vẫn chưa tạo/upload. Cần human sign-off mapping chưa rõ trước production.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" hidden="0" customHeight="1">
@@ -932,8 +932,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9c44c9bc8a24976"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R935b52edfa8a4516"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7d4e3947d1e48ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd16aa15779164bc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1337,10 +1337,10 @@
         <x:v>D:\Digiwin_Semiconducter_Workspace\ads\linkedin\LinkedIn_Build_Pack.md</x:v>
       </x:c>
       <x:c r="G18" s="42" t="str">
-        <x:v>Offline creative/build guidance is complete; no account/Page/placement proof.</x:v>
+        <x:v>Offline creative/build guidance complete; sanitized external validation completed on 2026-09-14. No delivery evidence.</x:v>
       </x:c>
       <x:c r="H18" s="42" t="str">
-        <x:v>Verify account, Page and placement through an authorized read-only UI review before any object work.</x:v>
+        <x:v>Human sign-off for unresolved entity mappings and an authorized production review remain required before any object work.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -1432,19 +1432,19 @@
         <x:v>Audience / retargeting</x:v>
       </x:c>
       <x:c r="D22" s="34" t="str">
-        <x:v>Planning draft — audience research</x:v>
+        <x:v>Planning draft — audience research and sanitized validation</x:v>
       </x:c>
       <x:c r="E22" s="34" t="str">
-        <x:v>Hoãn</x:v>
+        <x:v>Đang thực hiện</x:v>
       </x:c>
       <x:c r="F22" s="34" t="str">
         <x:v>D:\Digiwin_Semiconducter_Workspace\drafts\S03_LinkedIn_Audience_Research.md</x:v>
       </x:c>
       <x:c r="G22" s="42" t="str">
-        <x:v>Draft only; account/Page/audience eligibility not verified; no audience upload.</x:v>
+        <x:v>Sanitized external validation completed on 2026-09-14; raw account/audience evidence remains outside public Git. No upload, delivery or spend.</x:v>
       </x:c>
       <x:c r="H22" s="42" t="str">
-        <x:v>Audience and retargeting work is deferred by Bảo; no upload. Any future retargeting requires eligibility evidence (at least 300 reachable members).</x:v>
+        <x:v>Keep audience and retargeting uncreated. Require human sign-off for unresolved entity mappings and a separate mandate before production work.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" hidden="0" customHeight="1">
@@ -1638,7 +1638,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28dba6d7bf9d424d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8468c42fceef4816"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>